<commit_message>
Add threshold sensitivity and joint-genotyping check (manuscript v20)
</commit_message>
<xml_diff>
--- a/manuscript_v2/additional_files/Additional_file_5.xlsx
+++ b/manuscript_v2/additional_files/Additional_file_5.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tie-breaking" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PgTAGLip1-3 status" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primers (Table 8)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Threshold sensitivity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint genotyping" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +34,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -59,10 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="170" customWidth="1" min="1" max="1"/>
@@ -466,7 +475,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sheets: Ranking (all 184 loci); Tie-breaking; PgTAGLip1-3 status; Primers (Table 8).</t>
+          <t>Sheets: Ranking (all 184 loci); Tie-breaking; PgTAGLip1-3 status; Primers (Table 8); Threshold sensitivity; Joint genotyping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Threshold sensitivity</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Allele-level classes and panel selection under alternative paralog-cluster and complex-locus depth thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Joint genotyping</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Allele-level results and panel selection with both varieties genotyped jointly (robustness to the genotyping strategy).</t>
         </is>
       </c>
     </row>
@@ -787,7 +820,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -868,7 +900,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -917,7 +948,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -966,7 +996,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1015,7 +1044,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1064,7 +1092,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1107,7 +1134,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1150,7 +1176,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1193,7 +1218,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1242,7 +1266,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1285,7 +1308,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1328,7 +1350,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1371,7 +1392,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1543,7 +1563,6 @@
       <c r="U17" t="n">
         <v>2</v>
       </c>
-      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1586,7 +1605,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1635,7 +1653,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1716,7 +1733,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1797,7 +1813,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1872,7 +1887,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1947,7 +1961,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2028,7 +2041,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2071,7 +2083,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2114,7 +2125,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2157,7 +2167,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2200,7 +2209,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2243,7 +2251,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2286,7 +2293,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2335,7 +2341,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2378,7 +2383,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2427,7 +2431,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2476,7 +2479,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2525,7 +2527,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2697,7 +2698,6 @@
       <c r="U37" t="n">
         <v>2</v>
       </c>
-      <c r="V37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2781,7 +2781,6 @@
       <c r="U38" t="n">
         <v>3</v>
       </c>
-      <c r="V38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2865,7 +2864,6 @@
       <c r="U39" t="n">
         <v>4</v>
       </c>
-      <c r="V39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2949,7 +2947,6 @@
       <c r="U40" t="n">
         <v>5</v>
       </c>
-      <c r="V40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3033,7 +3030,6 @@
       <c r="U41" t="n">
         <v>6</v>
       </c>
-      <c r="V41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3117,7 +3113,6 @@
       <c r="U42" t="n">
         <v>7</v>
       </c>
-      <c r="V42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3201,7 +3196,6 @@
       <c r="U43" t="n">
         <v>8</v>
       </c>
-      <c r="V43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3285,7 +3279,6 @@
       <c r="U44" t="n">
         <v>9</v>
       </c>
-      <c r="V44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3369,7 +3362,6 @@
       <c r="U45" t="n">
         <v>10</v>
       </c>
-      <c r="V45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3453,7 +3445,6 @@
       <c r="U46" t="n">
         <v>11</v>
       </c>
-      <c r="V46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3537,7 +3528,6 @@
       <c r="U47" t="n">
         <v>12</v>
       </c>
-      <c r="V47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3621,7 +3611,6 @@
       <c r="U48" t="n">
         <v>13</v>
       </c>
-      <c r="V48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3705,7 +3694,6 @@
       <c r="U49" t="n">
         <v>14</v>
       </c>
-      <c r="V49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3789,7 +3777,6 @@
       <c r="U50" t="n">
         <v>15</v>
       </c>
-      <c r="V50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3873,7 +3860,6 @@
       <c r="U51" t="n">
         <v>16</v>
       </c>
-      <c r="V51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3957,7 +3943,6 @@
       <c r="U52" t="n">
         <v>17</v>
       </c>
-      <c r="V52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4041,7 +4026,6 @@
       <c r="U53" t="n">
         <v>18</v>
       </c>
-      <c r="V53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4125,7 +4109,6 @@
       <c r="U54" t="n">
         <v>19</v>
       </c>
-      <c r="V54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4209,7 +4192,6 @@
       <c r="U55" t="n">
         <v>20</v>
       </c>
-      <c r="V55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4293,7 +4275,6 @@
       <c r="U56" t="n">
         <v>21</v>
       </c>
-      <c r="V56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4377,7 +4358,6 @@
       <c r="U57" t="n">
         <v>22</v>
       </c>
-      <c r="V57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4461,7 +4441,6 @@
       <c r="U58" t="n">
         <v>23</v>
       </c>
-      <c r="V58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4545,7 +4524,6 @@
       <c r="U59" t="n">
         <v>24</v>
       </c>
-      <c r="V59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4629,7 +4607,6 @@
       <c r="U60" t="n">
         <v>25</v>
       </c>
-      <c r="V60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4713,7 +4690,6 @@
       <c r="U61" t="n">
         <v>26</v>
       </c>
-      <c r="V61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4797,7 +4773,6 @@
       <c r="U62" t="n">
         <v>27</v>
       </c>
-      <c r="V62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4881,7 +4856,6 @@
       <c r="U63" t="n">
         <v>28</v>
       </c>
-      <c r="V63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4965,7 +4939,6 @@
       <c r="U64" t="n">
         <v>29</v>
       </c>
-      <c r="V64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5049,7 +5022,6 @@
       <c r="U65" t="n">
         <v>30</v>
       </c>
-      <c r="V65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5133,7 +5105,6 @@
       <c r="U66" t="n">
         <v>31</v>
       </c>
-      <c r="V66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5214,7 +5185,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5295,7 +5265,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5376,7 +5345,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5457,7 +5425,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5538,7 +5505,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5613,7 +5579,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5694,7 +5659,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5775,7 +5739,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5856,7 +5819,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5937,7 +5899,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6018,7 +5979,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6099,7 +6059,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6180,7 +6139,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6261,7 +6219,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6342,7 +6299,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6423,7 +6379,6 @@
           <t>Excluded: complex locus (paralog-like cluster or &gt;2x depth)</t>
         </is>
       </c>
-      <c r="V82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6466,7 +6421,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6515,7 +6469,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6564,7 +6517,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6613,7 +6565,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6662,7 +6613,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6705,7 +6655,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6754,7 +6703,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6803,7 +6751,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6852,7 +6799,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6901,7 +6847,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6950,7 +6895,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6999,7 +6943,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7042,7 +6985,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7091,7 +7033,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7134,7 +7075,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7177,7 +7117,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7220,7 +7159,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7263,7 +7201,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7306,7 +7243,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7349,7 +7285,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7398,7 +7333,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7441,7 +7375,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7484,7 +7417,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7527,7 +7459,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7576,7 +7507,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7625,7 +7555,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7674,7 +7603,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7723,7 +7651,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7772,7 +7699,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7815,7 +7741,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7858,7 +7783,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7901,7 +7825,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7944,7 +7867,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7993,7 +7915,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8042,7 +7963,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8091,7 +8011,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8134,7 +8053,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8177,7 +8095,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8226,7 +8143,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8275,7 +8191,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8324,7 +8239,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8367,7 +8281,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8416,7 +8329,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8465,7 +8377,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -8508,7 +8419,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -8551,7 +8461,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8600,7 +8509,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8643,7 +8551,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -8686,7 +8593,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -8729,7 +8635,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -8772,7 +8677,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -8815,7 +8719,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -8858,7 +8761,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -8907,7 +8809,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -8956,7 +8857,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -8999,7 +8899,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9048,7 +8947,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -9097,7 +8995,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -9146,7 +9043,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -9195,7 +9091,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -9244,7 +9139,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -9293,7 +9187,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9342,7 +9235,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -9391,7 +9283,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -9440,7 +9331,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -9489,7 +9379,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -9532,7 +9421,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -9575,7 +9463,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -9618,7 +9505,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -9661,7 +9547,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -9710,7 +9595,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -9753,7 +9637,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -9796,7 +9679,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -9839,7 +9721,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -9882,7 +9763,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -9925,7 +9805,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -9968,7 +9847,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -10011,7 +9889,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -10054,7 +9931,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -10097,7 +9973,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -10140,7 +10015,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -10183,7 +10057,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -10226,7 +10099,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -10269,7 +10141,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -10318,7 +10189,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -10361,7 +10231,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -10410,7 +10279,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -10459,7 +10327,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -10508,7 +10375,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -10551,7 +10417,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -10594,7 +10459,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -10637,7 +10501,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -10686,7 +10549,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -10729,7 +10591,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -10810,7 +10671,6 @@
           <t>Excluded: truncated gene model (&lt;70% of best-hit length)</t>
         </is>
       </c>
-      <c r="V177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -10853,7 +10713,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -10902,7 +10761,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -10945,7 +10803,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -10988,7 +10845,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -11037,7 +10893,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -11080,7 +10935,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -11123,7 +10977,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -11166,7 +11019,6 @@
           <t>No validated variety-specific coding allele</t>
         </is>
       </c>
-      <c r="V185" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11897,4 +11749,2562 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Sensitivity of the allele-level classification and panel selection to the a priori paralog-cluster and complex-locus depth thresholds (one threshold changed at a time; all other thresholds as in Methods 5.6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Change from baseline</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Paralog-flagged coding alleles</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Validated specific alleles, GHB-732</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Validated specific alleles, GHB-538</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Reliable alleles without read-level data</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>LR-specific genes</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>HR-specific genes</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Genes with specific alleles in each variety</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Complex loci</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Eligible scored loci</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Selected TAG lipase</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Selected MAG lipase</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Selected class III peroxidase</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>≥4 calls, AF&lt;0.35, 100 bp; depth &gt;2×</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2405</v>
+      </c>
+      <c r="D3" t="n">
+        <v>418</v>
+      </c>
+      <c r="E3" t="n">
+        <v>257</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>142</v>
+      </c>
+      <c r="H3" t="n">
+        <v>83</v>
+      </c>
+      <c r="I3" t="n">
+        <v>41</v>
+      </c>
+      <c r="J3" t="n">
+        <v>283</v>
+      </c>
+      <c r="K3" t="n">
+        <v>34</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>K=3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>≥3 calls</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2867</v>
+      </c>
+      <c r="D4" t="n">
+        <v>390</v>
+      </c>
+      <c r="E4" t="n">
+        <v>241</v>
+      </c>
+      <c r="F4" t="n">
+        <v>72</v>
+      </c>
+      <c r="G4" t="n">
+        <v>121</v>
+      </c>
+      <c r="H4" t="n">
+        <v>71</v>
+      </c>
+      <c r="I4" t="n">
+        <v>32</v>
+      </c>
+      <c r="J4" t="n">
+        <v>386</v>
+      </c>
+      <c r="K4" t="n">
+        <v>31</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>POX Pgl_GLEAN_10004812</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>K=5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>≥5 calls</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D5" t="n">
+        <v>418</v>
+      </c>
+      <c r="E5" t="n">
+        <v>257</v>
+      </c>
+      <c r="F5" t="n">
+        <v>92</v>
+      </c>
+      <c r="G5" t="n">
+        <v>155</v>
+      </c>
+      <c r="H5" t="n">
+        <v>90</v>
+      </c>
+      <c r="I5" t="n">
+        <v>44</v>
+      </c>
+      <c r="J5" t="n">
+        <v>225</v>
+      </c>
+      <c r="K5" t="n">
+        <v>35</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AF&lt;0.30</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AF &lt;0.30</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1912</v>
+      </c>
+      <c r="D6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E6" t="n">
+        <v>257</v>
+      </c>
+      <c r="F6" t="n">
+        <v>283</v>
+      </c>
+      <c r="G6" t="n">
+        <v>145</v>
+      </c>
+      <c r="H6" t="n">
+        <v>87</v>
+      </c>
+      <c r="I6" t="n">
+        <v>43</v>
+      </c>
+      <c r="J6" t="n">
+        <v>257</v>
+      </c>
+      <c r="K6" t="n">
+        <v>35</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AF&lt;0.40</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AF &lt;0.40</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2854</v>
+      </c>
+      <c r="D7" t="n">
+        <v>395</v>
+      </c>
+      <c r="E7" t="n">
+        <v>231</v>
+      </c>
+      <c r="F7" t="n">
+        <v>137</v>
+      </c>
+      <c r="G7" t="n">
+        <v>133</v>
+      </c>
+      <c r="H7" t="n">
+        <v>77</v>
+      </c>
+      <c r="I7" t="n">
+        <v>39</v>
+      </c>
+      <c r="J7" t="n">
+        <v>312</v>
+      </c>
+      <c r="K7" t="n">
+        <v>33</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>none eligible (SDP1 classed as complex locus)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>W=50bp</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>50-bp window</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2049</v>
+      </c>
+      <c r="D8" t="n">
+        <v>418</v>
+      </c>
+      <c r="E8" t="n">
+        <v>257</v>
+      </c>
+      <c r="F8" t="n">
+        <v>89</v>
+      </c>
+      <c r="G8" t="n">
+        <v>154</v>
+      </c>
+      <c r="H8" t="n">
+        <v>90</v>
+      </c>
+      <c r="I8" t="n">
+        <v>43</v>
+      </c>
+      <c r="J8" t="n">
+        <v>239</v>
+      </c>
+      <c r="K8" t="n">
+        <v>36</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>W=200bp</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>200-bp window</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2724</v>
+      </c>
+      <c r="D9" t="n">
+        <v>395</v>
+      </c>
+      <c r="E9" t="n">
+        <v>247</v>
+      </c>
+      <c r="F9" t="n">
+        <v>51</v>
+      </c>
+      <c r="G9" t="n">
+        <v>128</v>
+      </c>
+      <c r="H9" t="n">
+        <v>78</v>
+      </c>
+      <c r="I9" t="n">
+        <v>39</v>
+      </c>
+      <c r="J9" t="n">
+        <v>326</v>
+      </c>
+      <c r="K9" t="n">
+        <v>32</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>POX Pgl_GLEAN_10004812</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>depth&gt;1.5x</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>depth &gt;1.5× median</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2405</v>
+      </c>
+      <c r="D10" t="n">
+        <v>418</v>
+      </c>
+      <c r="E10" t="n">
+        <v>257</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>124</v>
+      </c>
+      <c r="H10" t="n">
+        <v>76</v>
+      </c>
+      <c r="I10" t="n">
+        <v>37</v>
+      </c>
+      <c r="J10" t="n">
+        <v>396</v>
+      </c>
+      <c r="K10" t="n">
+        <v>31</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>depth&gt;3x</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>depth &gt;3× median</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2405</v>
+      </c>
+      <c r="D11" t="n">
+        <v>418</v>
+      </c>
+      <c r="E11" t="n">
+        <v>257</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>143</v>
+      </c>
+      <c r="H11" t="n">
+        <v>83</v>
+      </c>
+      <c r="I11" t="n">
+        <v>41</v>
+      </c>
+      <c r="J11" t="n">
+        <v>270</v>
+      </c>
+      <c r="K11" t="n">
+        <v>34</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Note: alleles that became reliable, or lost their "shared" status, only under an alternative setting were not re-checked in the BAM files and were counted as not validated; counts of validated alleles under looser settings are therefore lower bounds. Panel selection: MAGL selected in 9/9 settings, SDP1 in 8/9 and the PER52-like peroxidase in 7/9.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M70"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Robustness of the allele-level comparison to the genotyping strategy: published analysis (per-sample genotyping of each variety) versus joint genotyping of both varieties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Joint call set: GATK 4.6.2.0 HaplotypeCaller (-ERC GVCF) on both final BAM files over the 1,370 gene models (mRNA ± 100 bp; interval padding 100 bp), CombineGVCFs and GenotypeGVCFs; same SNP/INDEL hard filters, SnpEff 5.3 annotation, reliability, paralog-cluster, read-level and complex-locus rules as Methods 5.3–5.6. Absence in the other variety was taken from that variety's joint genotype (called genotype, read depth ≥ 10). Read counts were obtained for the 53 sites not inspected in the published analysis; 12 previously inspected sites re-counted as controls gave identical counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Published analysis</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Joint genotyping</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Validated variety-specific alleles, GHB-732</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>418</v>
+      </c>
+      <c r="C5" t="n">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Validated variety-specific alleles, GHB-538</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>257</v>
+      </c>
+      <c r="C6" t="n">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Validated alleles identical in both analyses</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>672 of 675</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LR-specific genes</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>142</v>
+      </c>
+      <c r="C8" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HR-specific genes</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>83</v>
+      </c>
+      <c r="C9" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Genes with specific alleles in each variety</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>41</v>
+      </c>
+      <c r="C10" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Complex loci</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>283</v>
+      </c>
+      <c r="C11" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Genes with the same allele-level class</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1,340 of 1,370 (97.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Eligible scored loci</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>34</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>34 (33 identical)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Selected TAG lipase</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Selected MAG lipase</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Selected class III peroxidase</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PER52-like POX (Pgl_GLEAN_10033116)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170); Pgl_GLEAN_10033116 becomes a complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Threshold sensitivity on the joint call set (settings as in sheet "Threshold sensitivity")</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Paralog-flagged coding alleles</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Validated specific alleles, GHB-732</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Validated specific alleles, GHB-538</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Reliable alleles without read-level data</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>LR-specific genes</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>HR-specific genes</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Genes with specific alleles in each variety</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Complex loci</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Eligible scored loci</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Selected TAG lipase</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Selected MAG lipase</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Selected class III peroxidase</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2561</v>
+      </c>
+      <c r="C20" t="n">
+        <v>418</v>
+      </c>
+      <c r="D20" t="n">
+        <v>257</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>141</v>
+      </c>
+      <c r="G20" t="n">
+        <v>83</v>
+      </c>
+      <c r="H20" t="n">
+        <v>37</v>
+      </c>
+      <c r="I20" t="n">
+        <v>290</v>
+      </c>
+      <c r="J20" t="n">
+        <v>34</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>K=3</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3083</v>
+      </c>
+      <c r="C21" t="n">
+        <v>390</v>
+      </c>
+      <c r="D21" t="n">
+        <v>241</v>
+      </c>
+      <c r="E21" t="n">
+        <v>68</v>
+      </c>
+      <c r="F21" t="n">
+        <v>118</v>
+      </c>
+      <c r="G21" t="n">
+        <v>70</v>
+      </c>
+      <c r="H21" t="n">
+        <v>29</v>
+      </c>
+      <c r="I21" t="n">
+        <v>395</v>
+      </c>
+      <c r="J21" t="n">
+        <v>29</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>POX Pgl_GLEAN_10004812</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>K=5</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2175</v>
+      </c>
+      <c r="C22" t="n">
+        <v>419</v>
+      </c>
+      <c r="D22" t="n">
+        <v>257</v>
+      </c>
+      <c r="E22" t="n">
+        <v>78</v>
+      </c>
+      <c r="F22" t="n">
+        <v>157</v>
+      </c>
+      <c r="G22" t="n">
+        <v>89</v>
+      </c>
+      <c r="H22" t="n">
+        <v>44</v>
+      </c>
+      <c r="I22" t="n">
+        <v>230</v>
+      </c>
+      <c r="J22" t="n">
+        <v>37</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AF&lt;0.30</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2056</v>
+      </c>
+      <c r="C23" t="n">
+        <v>419</v>
+      </c>
+      <c r="D23" t="n">
+        <v>257</v>
+      </c>
+      <c r="E23" t="n">
+        <v>279</v>
+      </c>
+      <c r="F23" t="n">
+        <v>146</v>
+      </c>
+      <c r="G23" t="n">
+        <v>87</v>
+      </c>
+      <c r="H23" t="n">
+        <v>38</v>
+      </c>
+      <c r="I23" t="n">
+        <v>266</v>
+      </c>
+      <c r="J23" t="n">
+        <v>37</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AF&lt;0.40</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3027</v>
+      </c>
+      <c r="C24" t="n">
+        <v>394</v>
+      </c>
+      <c r="D24" t="n">
+        <v>231</v>
+      </c>
+      <c r="E24" t="n">
+        <v>137</v>
+      </c>
+      <c r="F24" t="n">
+        <v>133</v>
+      </c>
+      <c r="G24" t="n">
+        <v>77</v>
+      </c>
+      <c r="H24" t="n">
+        <v>35</v>
+      </c>
+      <c r="I24" t="n">
+        <v>315</v>
+      </c>
+      <c r="J24" t="n">
+        <v>33</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>none (SDP1 becomes a complex locus)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>W=50bp</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2151</v>
+      </c>
+      <c r="C25" t="n">
+        <v>418</v>
+      </c>
+      <c r="D25" t="n">
+        <v>257</v>
+      </c>
+      <c r="E25" t="n">
+        <v>82</v>
+      </c>
+      <c r="F25" t="n">
+        <v>152</v>
+      </c>
+      <c r="G25" t="n">
+        <v>89</v>
+      </c>
+      <c r="H25" t="n">
+        <v>43</v>
+      </c>
+      <c r="I25" t="n">
+        <v>243</v>
+      </c>
+      <c r="J25" t="n">
+        <v>36</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>W=200bp</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2947</v>
+      </c>
+      <c r="C26" t="n">
+        <v>395</v>
+      </c>
+      <c r="D26" t="n">
+        <v>247</v>
+      </c>
+      <c r="E26" t="n">
+        <v>55</v>
+      </c>
+      <c r="F26" t="n">
+        <v>129</v>
+      </c>
+      <c r="G26" t="n">
+        <v>77</v>
+      </c>
+      <c r="H26" t="n">
+        <v>34</v>
+      </c>
+      <c r="I26" t="n">
+        <v>337</v>
+      </c>
+      <c r="J26" t="n">
+        <v>33</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>depth&gt;1.5x</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2561</v>
+      </c>
+      <c r="C27" t="n">
+        <v>418</v>
+      </c>
+      <c r="D27" t="n">
+        <v>257</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G27" t="n">
+        <v>75</v>
+      </c>
+      <c r="H27" t="n">
+        <v>33</v>
+      </c>
+      <c r="I27" t="n">
+        <v>404</v>
+      </c>
+      <c r="J27" t="n">
+        <v>30</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>depth&gt;3x</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2561</v>
+      </c>
+      <c r="C28" t="n">
+        <v>418</v>
+      </c>
+      <c r="D28" t="n">
+        <v>257</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>142</v>
+      </c>
+      <c r="G28" t="n">
+        <v>83</v>
+      </c>
+      <c r="H28" t="n">
+        <v>37</v>
+      </c>
+      <c r="I28" t="n">
+        <v>278</v>
+      </c>
+      <c r="J28" t="n">
+        <v>34</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>SDP1 (Pgl_GLEAN_10017888)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>MAGL (Pgl_GLEAN_10036216)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>PER66-like POX (Pgl_GLEAN_10011170)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Validated alleles that differ between the analyses</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Variety</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Chromosome</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Alt</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Protein change</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Published analysis</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Joint genotyping</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GHB-732</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10005891</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>chr6</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>15368112</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>p.Ile312Asn</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>specific</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>not reliable</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>allele fraction 0.25 → 0.19 after re-genotyping</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GHB-732</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10033116</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>chr3</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>202355236</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>p.Ser180fs</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>specific</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>not reliable</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>in a paralog-like cluster after joint calling added low-fraction calls</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>GHB-732</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10033968</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>chr4</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>76211371</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>p.Gln22Pro</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>specific</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>not called</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>not called in the joint call set</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>GHB-732</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10018093</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>chr2</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>242184113</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>p.Cys13Trp</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>not reliable (paralog-like)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>specific</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>paralog-like cluster not reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>GHB-732</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10028026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>chr3</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>226832433</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>p.Gly205Arg</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>not reliable (paralog-like)</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>specific</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>paralog-like cluster not reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>GHB-732</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10037756</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>chr5</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>156071863</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>p.Ala307Thr</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>not reliable</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>specific</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>allele fraction 0.24 → 0.26 after re-genotyping</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Genes whose allele-level class differs between the analyses</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Functional category</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Annotation</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Published analysis</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Joint genotyping</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10000530</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>sp|Q6RYA0|SABP2_TOBAC</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>No reliable coding difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10005892</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>sp|Q9M084|SYDC2_ARATH</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Both varieties</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10006486</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>sp|A7QEU4|PER5_VITVI Peroxidase 5 OS=Vitis vinifera OX=29760 GN=GSVIVT00037159001 PE=1 SV=2</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10011135</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>sp|P93733|PLDB1_ARATH Phospholipase D beta 1 OS=Arabidopsis thaliana OX=3702 GN=PLDBETA1 PE=1 SV=4</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10011170</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>sp|A5H454|PER66_MAIZE Peroxidase 66 OS=Zea mays OX=4577 GN=PER66 PE=1 SV=1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LR-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10011172</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>sp|Q0D3N0|PER2_ORYSJ Peroxidase 2 OS=Oryza sativa subsp. japonica OX=39947 GN=PRX112 PE=2 SV=1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10012151</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>A0A9D4A6K3_9ROSI</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Both varieties</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10012869</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>sp|B4FZ87|ACHE_MAIZE GDSL esterase/lipase ACHE OS=Zea mays OX=4577 GN=ACHE PE=1 SV=1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10013636</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Aldehyde/alcohol metabolism</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>A0A368QGF6_SETIT Allyl alcohol dehydrogenase-like protein {ECO:0008006|Google:ProtNLM}</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10017594</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>sp|Q7G4G7|AT1_ORYSJ</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>LR-specific</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10018093</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>sp|Q9ZPQ3|GEK1_ARATH</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LR-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10018694</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>sp|Q53QK0|Y1103_ORYSJ</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10019127</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>sp|Q9FJ45|GDL83_ARATH GDSL esterase/lipase At5g45910 OS=Arabidopsis thaliana OX=3702 GN=At5g45910 PE=2 SV=1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>No reliable coding difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10019327</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>sp|P84516|PER1_SORBI Cationic peroxidase SPC4 OS=Sorghum bicolor OX=4558 GN=Sb03g046810 PE=1 SV=2</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>No reliable coding difference</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10020403</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>sp|Q9THX6|TL29_SOLLC</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10021899</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>sp|Q9FG34|PER54_ARATH Peroxidase 54 OS=Arabidopsis thaliana OX=3702 GN=PER54 PE=2 SV=1</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Both varieties</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10022802</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>sp|Q9LT10|CXE18_ARATH Probable carboxylesterase 18 OS=Arabidopsis thaliana OX=3702 GN=CXE18 PE=1 SV=1</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>HR-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10023543</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>sp|A0AAW1NHX6|SDR1_SAPOF</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>No reliable coding difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10024393</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>sp|P0DXJ4|AAE1_RAUSE Acetylajmalan esterase 1 OS=Rauvolfia serpentina OX=4060 GN=AAE1 PE=1 SV=1</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10025566</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>sp|Q67ZI9|GDL48_ARATH GDSL esterase/lipase At2g42990 OS=Arabidopsis thaliana OX=3702 GN=At2g42990 PE=2 SV=1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>HR-specific</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10026548</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>sp|O80522|GDL2_ARATH GDSL esterase/lipase At1g09390 OS=Arabidopsis thaliana OX=3702 GN=At1g09390 PE=2 SV=1</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>No reliable coding difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10030100</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>sp|Q6KAJ8|RL391_ORYSJ</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>No reliable coding difference</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10032394</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Lipid oxidation / oxygenase</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>sp|P29250|LOX2_ORYSJ Linoleate 9S-lipoxygenase 2 OS=Oryza sativa subsp. japonica OX=39947 GN=LOX1.1 PE=2 SV=2</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10032687</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Phenolic / secondary oxidative metabolism</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>sp|Q0JBZ8|HCT1_ORYSJ</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>No reliable coding difference</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10033116</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>sp|Q9FLC0|PER52_ARATH Peroxidase 52 OS=Arabidopsis thaliana OX=3702 GN=PER52 PE=2 SV=1</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>LR-specific</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10035569</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Not assigned (auxiliary/other)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>sp|P22989|LDHB_HORVU</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10036318</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>sp|Q9FJ45|GDL83_ARATH GDSL esterase/lipase At5g45910 OS=Arabidopsis thaliana OX=3702 GN=At5g45910 PE=2 SV=1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10037522</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Phenolic / secondary oxidative metabolism</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>sp|A8QW53|OMT3_SORBI</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Both varieties</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10037553</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Oxidative defence / redox</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>sp|P0DKC5|HSD1A_ARATH</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>LR-specific</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Pgl_GLEAN_10038272</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Lipid hydrolysis</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>sp|B4FZ87|ACHE_MAIZE GDSL esterase/lipase ACHE OS=Zea mays OX=4577 GN=ACHE PE=1 SV=1</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Shared alleles only</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Complex locus</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>